<commit_message>
Update KPIs and run experiments
</commit_message>
<xml_diff>
--- a/inputData/LTM_demand5min.xlsx
+++ b/inputData/LTM_demand5min.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,16 +465,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -491,10 +491,10 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -505,19 +505,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>69</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -525,16 +525,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -545,16 +545,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -568,10 +568,10 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
@@ -588,16 +588,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -611,10 +611,10 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -625,16 +625,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -651,10 +651,10 @@
         <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -665,19 +665,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -685,19 +685,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -705,19 +705,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -725,16 +725,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
@@ -745,19 +745,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -765,13 +765,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
@@ -791,10 +791,10 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>167</v>
+        <v>146</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -805,13 +805,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>173</v>
+        <v>147</v>
       </c>
       <c r="E19" t="n">
         <v>3</v>
@@ -825,16 +825,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>187</v>
+        <v>153</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
@@ -845,19 +845,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>235</v>
+        <v>196</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -865,16 +865,16 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>401</v>
+        <v>200</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -888,16 +888,16 @@
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>461</v>
+        <v>382</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -905,16 +905,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>510</v>
+        <v>411</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -925,16 +925,16 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>510</v>
+        <v>462</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -945,16 +945,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>521</v>
+        <v>493</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -965,10 +965,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
         <v>521</v>
@@ -985,16 +985,16 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1008,13 +1008,13 @@
         <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1025,19 +1025,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="E30" t="n">
         <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1045,13 +1045,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>531</v>
+        <v>538</v>
       </c>
       <c r="E31" t="n">
         <v>3</v>
@@ -1065,19 +1065,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D32" t="n">
-        <v>546</v>
+        <v>554</v>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -1085,19 +1085,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C33" t="n">
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1105,19 +1105,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>576</v>
+        <v>559</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1125,16 +1125,16 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D35" t="n">
-        <v>607</v>
+        <v>559</v>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -1145,13 +1145,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>615</v>
+        <v>577</v>
       </c>
       <c r="E36" t="n">
         <v>4</v>
@@ -1168,13 +1168,13 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>632</v>
+        <v>579</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -1185,13 +1185,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D38" t="n">
-        <v>632</v>
+        <v>586</v>
       </c>
       <c r="E38" t="n">
         <v>3</v>
@@ -1211,13 +1211,13 @@
         <v>1</v>
       </c>
       <c r="D39" t="n">
-        <v>633</v>
+        <v>591</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1225,19 +1225,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D40" t="n">
-        <v>639</v>
+        <v>594</v>
       </c>
       <c r="E40" t="n">
         <v>4</v>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1245,16 +1245,16 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>659</v>
+        <v>596</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -1265,19 +1265,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>692</v>
+        <v>614</v>
       </c>
       <c r="E42" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -1285,16 +1285,16 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>697</v>
+        <v>640</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
@@ -1311,7 +1311,7 @@
         <v>2</v>
       </c>
       <c r="D44" t="n">
-        <v>701</v>
+        <v>643</v>
       </c>
       <c r="E44" t="n">
         <v>2</v>
@@ -1331,13 +1331,53 @@
         <v>4</v>
       </c>
       <c r="D45" t="n">
-        <v>741</v>
+        <v>667</v>
       </c>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="n">
+        <v>681</v>
+      </c>
+      <c r="E46" t="n">
+        <v>4</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>723</v>
+      </c>
+      <c r="E47" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Let eVTOL charge in the first operation in Heuristic
</commit_message>
<xml_diff>
--- a/inputData/LTM_demand5min.xlsx
+++ b/inputData/LTM_demand5min.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,16 +465,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -491,13 +491,13 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -511,13 +511,13 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -525,19 +525,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -545,19 +545,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C6" t="n">
         <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -565,19 +565,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -585,16 +585,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
@@ -605,19 +605,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -628,13 +628,13 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -648,13 +648,13 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -665,19 +665,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -685,19 +685,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -705,16 +705,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -731,10 +731,10 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
@@ -751,10 +751,10 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
@@ -765,19 +765,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -785,19 +785,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -805,16 +805,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -831,10 +831,10 @@
         <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
@@ -851,13 +851,13 @@
         <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>196</v>
+        <v>155</v>
       </c>
       <c r="E21" t="n">
         <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -865,19 +865,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>200</v>
+        <v>167</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -885,19 +885,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C23" t="n">
         <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>382</v>
+        <v>189</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -908,13 +908,13 @@
         <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>411</v>
+        <v>204</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -925,19 +925,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" t="n">
-        <v>462</v>
+        <v>208</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -945,16 +945,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>493</v>
+        <v>374</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -965,19 +965,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D27" t="n">
-        <v>521</v>
+        <v>391</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -991,13 +991,13 @@
         <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>524</v>
+        <v>394</v>
       </c>
       <c r="E28" t="n">
         <v>4</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1005,16 +1005,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>527</v>
+        <v>399</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1025,16 +1025,16 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>536</v>
+        <v>418</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
@@ -1045,13 +1045,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D31" t="n">
-        <v>538</v>
+        <v>431</v>
       </c>
       <c r="E31" t="n">
         <v>3</v>
@@ -1065,19 +1065,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>554</v>
+        <v>472</v>
       </c>
       <c r="E32" t="n">
         <v>4</v>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -1091,7 +1091,7 @@
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>559</v>
+        <v>472</v>
       </c>
       <c r="E33" t="n">
         <v>3</v>
@@ -1105,13 +1105,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>559</v>
+        <v>530</v>
       </c>
       <c r="E34" t="n">
         <v>1</v>
@@ -1128,16 +1128,16 @@
         <v>4</v>
       </c>
       <c r="C35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1148,10 +1148,10 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>577</v>
+        <v>567</v>
       </c>
       <c r="E36" t="n">
         <v>4</v>
@@ -1165,13 +1165,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>579</v>
+        <v>574</v>
       </c>
       <c r="E37" t="n">
         <v>2</v>
@@ -1185,16 +1185,16 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -1205,19 +1205,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D39" t="n">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -1225,19 +1225,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D40" t="n">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -1245,19 +1245,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C41" t="n">
         <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -1265,16 +1265,16 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D42" t="n">
-        <v>614</v>
+        <v>606</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
         <v>1</v>
@@ -1285,19 +1285,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
-        <v>640</v>
+        <v>620</v>
       </c>
       <c r="E43" t="n">
         <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -1305,19 +1305,19 @@
         <v>43</v>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>643</v>
+        <v>629</v>
       </c>
       <c r="E44" t="n">
         <v>2</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -1325,16 +1325,16 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>667</v>
+        <v>631</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
@@ -1345,16 +1345,16 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>681</v>
+        <v>637</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
         <v>1</v>
@@ -1371,13 +1371,53 @@
         <v>2</v>
       </c>
       <c r="D47" t="n">
-        <v>723</v>
+        <v>686</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="n">
+        <v>720</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" t="n">
+        <v>732</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Experimental study, also added output to heuristic func to return profit (obj + "penaties from battery and passengers)
</commit_message>
<xml_diff>
--- a/inputData/LTM_demand5min.xlsx
+++ b/inputData/LTM_demand5min.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,19 +465,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E2" t="n">
         <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -491,10 +491,10 @@
         <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -505,19 +505,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
         <v>71</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -525,19 +525,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -545,19 +545,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -568,13 +568,13 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -585,19 +585,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>104</v>
+        <v>140</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -608,16 +608,16 @@
         <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -628,13 +628,13 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>117</v>
+        <v>146</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -648,16 +648,16 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -665,16 +665,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>137</v>
+        <v>192</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -688,16 +688,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>142</v>
+        <v>201</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -705,16 +705,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>152</v>
+        <v>416</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
@@ -725,19 +725,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>164</v>
+        <v>431</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -745,13 +745,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>170</v>
+        <v>432</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
@@ -765,19 +765,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
-        <v>174</v>
+        <v>478</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -785,19 +785,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>401</v>
+        <v>485</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -811,10 +811,10 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>411</v>
+        <v>486</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -828,13 +828,13 @@
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>413</v>
+        <v>511</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -845,19 +845,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
         <v>5</v>
       </c>
-      <c r="C21" t="n">
-        <v>2</v>
-      </c>
       <c r="D21" t="n">
-        <v>459</v>
+        <v>518</v>
       </c>
       <c r="E21" t="n">
         <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -868,13 +868,13 @@
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>464</v>
+        <v>522</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -885,16 +885,16 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>515</v>
+        <v>529</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -911,10 +911,10 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>515</v>
+        <v>541</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -925,19 +925,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>520</v>
+        <v>564</v>
       </c>
       <c r="E25" t="n">
         <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -945,16 +945,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>529</v>
+        <v>588</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -965,16 +965,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>538</v>
+        <v>602</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
         <v>1</v>
@@ -985,16 +985,16 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>541</v>
+        <v>676</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F28" t="n">
         <v>1</v>
@@ -1005,19 +1005,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>541</v>
+        <v>722</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1025,338 +1025,18 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D30" t="n">
-        <v>548</v>
+        <v>745</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>4</v>
-      </c>
-      <c r="D31" t="n">
-        <v>566</v>
-      </c>
-      <c r="E31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F31" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" t="n">
-        <v>2</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>580</v>
-      </c>
-      <c r="E32" t="n">
-        <v>4</v>
-      </c>
-      <c r="F32" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" t="n">
-        <v>2</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
-        <v>583</v>
-      </c>
-      <c r="E33" t="n">
-        <v>3</v>
-      </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" t="n">
-        <v>4</v>
-      </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" t="n">
-        <v>589</v>
-      </c>
-      <c r="E34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" t="n">
-        <v>5</v>
-      </c>
-      <c r="C35" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" t="n">
-        <v>598</v>
-      </c>
-      <c r="E35" t="n">
-        <v>2</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>4</v>
-      </c>
-      <c r="D36" t="n">
-        <v>604</v>
-      </c>
-      <c r="E36" t="n">
-        <v>4</v>
-      </c>
-      <c r="F36" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>3</v>
-      </c>
-      <c r="D37" t="n">
-        <v>609</v>
-      </c>
-      <c r="E37" t="n">
-        <v>2</v>
-      </c>
-      <c r="F37" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" t="n">
-        <v>2</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
-        <v>620</v>
-      </c>
-      <c r="E38" t="n">
-        <v>2</v>
-      </c>
-      <c r="F38" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" t="n">
-        <v>2</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="n">
-        <v>624</v>
-      </c>
-      <c r="E39" t="n">
-        <v>2</v>
-      </c>
-      <c r="F39" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>2</v>
-      </c>
-      <c r="D40" t="n">
-        <v>627</v>
-      </c>
-      <c r="E40" t="n">
-        <v>2</v>
-      </c>
-      <c r="F40" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>4</v>
-      </c>
-      <c r="D41" t="n">
-        <v>627</v>
-      </c>
-      <c r="E41" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
-        <v>636</v>
-      </c>
-      <c r="E42" t="n">
-        <v>2</v>
-      </c>
-      <c r="F42" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" t="n">
-        <v>650</v>
-      </c>
-      <c r="E43" t="n">
-        <v>4</v>
-      </c>
-      <c r="F43" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" t="n">
-        <v>2</v>
-      </c>
-      <c r="D44" t="n">
-        <v>655</v>
-      </c>
-      <c r="E44" t="n">
-        <v>3</v>
-      </c>
-      <c r="F44" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" t="n">
-        <v>4</v>
-      </c>
-      <c r="C45" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" t="n">
-        <v>658</v>
-      </c>
-      <c r="E45" t="n">
-        <v>4</v>
-      </c>
-      <c r="F45" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="n">
-        <v>4</v>
-      </c>
-      <c r="D46" t="n">
-        <v>713</v>
-      </c>
-      <c r="E46" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Clean up and data changes
</commit_message>
<xml_diff>
--- a/inputData/LTM_demand5min.xlsx
+++ b/inputData/LTM_demand5min.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,16 +465,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
         <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -488,16 +488,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -505,19 +505,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -525,16 +525,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -545,16 +545,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -565,19 +565,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -585,16 +585,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>140</v>
+        <v>89</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
@@ -605,16 +605,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>143</v>
+        <v>91</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
@@ -628,13 +628,13 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D10" t="n">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -645,19 +645,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>185</v>
+        <v>94</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -665,19 +665,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>192</v>
+        <v>99</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -685,19 +685,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>201</v>
+        <v>100</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -705,19 +705,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D14" t="n">
-        <v>416</v>
+        <v>101</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -728,16 +728,16 @@
         <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>431</v>
+        <v>103</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -748,13 +748,13 @@
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>432</v>
+        <v>103</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
@@ -765,16 +765,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>478</v>
+        <v>108</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -785,13 +785,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>485</v>
+        <v>109</v>
       </c>
       <c r="E18" t="n">
         <v>3</v>
@@ -808,13 +808,13 @@
         <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D19" t="n">
-        <v>486</v>
+        <v>110</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -825,16 +825,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
-        <v>511</v>
+        <v>111</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -848,16 +848,16 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>518</v>
+        <v>113</v>
       </c>
       <c r="E21" t="n">
         <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -865,19 +865,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>522</v>
+        <v>116</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -888,16 +888,16 @@
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D23" t="n">
-        <v>529</v>
+        <v>126</v>
       </c>
       <c r="E23" t="n">
         <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -905,19 +905,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>541</v>
+        <v>141</v>
       </c>
       <c r="E24" t="n">
         <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -925,13 +925,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>564</v>
+        <v>147</v>
       </c>
       <c r="E25" t="n">
         <v>4</v>
@@ -945,16 +945,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C26" t="n">
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>588</v>
+        <v>148</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -965,16 +965,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="n">
         <v>2</v>
       </c>
-      <c r="C27" t="n">
-        <v>1</v>
-      </c>
       <c r="D27" t="n">
-        <v>602</v>
+        <v>150</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
         <v>1</v>
@@ -985,19 +985,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D28" t="n">
-        <v>676</v>
+        <v>152</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1005,16 +1005,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D29" t="n">
-        <v>722</v>
+        <v>153</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1025,18 +1025,598 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C30" t="n">
+        <v>7</v>
+      </c>
+      <c r="D30" t="n">
+        <v>154</v>
+      </c>
+      <c r="E30" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>7</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>156</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>161</v>
+      </c>
+      <c r="E32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" t="n">
+        <v>8</v>
+      </c>
+      <c r="D33" t="n">
+        <v>172</v>
+      </c>
+      <c r="E33" t="n">
+        <v>4</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>8</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>180</v>
+      </c>
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>7</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>186</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>9</v>
+      </c>
+      <c r="D36" t="n">
+        <v>186</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>189</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>7</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>204</v>
+      </c>
+      <c r="E38" t="n">
+        <v>4</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D39" t="n">
+        <v>215</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>344</v>
+      </c>
+      <c r="E40" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>6</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>451</v>
+      </c>
+      <c r="E41" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" t="n">
+        <v>10</v>
+      </c>
+      <c r="D42" t="n">
+        <v>480</v>
+      </c>
+      <c r="E42" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>10</v>
+      </c>
+      <c r="C43" t="n">
         <v>5</v>
       </c>
-      <c r="D30" t="n">
-        <v>745</v>
-      </c>
-      <c r="E30" t="n">
-        <v>3</v>
-      </c>
-      <c r="F30" t="n">
+      <c r="D43" t="n">
+        <v>509</v>
+      </c>
+      <c r="E43" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>7</v>
+      </c>
+      <c r="C44" t="n">
+        <v>3</v>
+      </c>
+      <c r="D44" t="n">
+        <v>510</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>7</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>518</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>7</v>
+      </c>
+      <c r="D46" t="n">
+        <v>543</v>
+      </c>
+      <c r="E46" t="n">
+        <v>4</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>9</v>
+      </c>
+      <c r="D47" t="n">
+        <v>557</v>
+      </c>
+      <c r="E47" t="n">
+        <v>4</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>8</v>
+      </c>
+      <c r="C48" t="n">
+        <v>7</v>
+      </c>
+      <c r="D48" t="n">
+        <v>558</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>561</v>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="n">
+        <v>7</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>585</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>9</v>
+      </c>
+      <c r="D51" t="n">
+        <v>591</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="n">
+        <v>10</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="n">
+        <v>595</v>
+      </c>
+      <c r="E52" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="n">
+        <v>7</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>604</v>
+      </c>
+      <c r="E53" t="n">
+        <v>3</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>7</v>
+      </c>
+      <c r="D54" t="n">
+        <v>622</v>
+      </c>
+      <c r="E54" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="n">
+        <v>7</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>625</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="n">
+        <v>8</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>627</v>
+      </c>
+      <c r="E56" t="n">
+        <v>4</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>9</v>
+      </c>
+      <c r="D57" t="n">
+        <v>642</v>
+      </c>
+      <c r="E57" t="n">
+        <v>3</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="n">
+        <v>7</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>702</v>
+      </c>
+      <c r="E58" t="n">
+        <v>3</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="n">
+        <v>7</v>
+      </c>
+      <c r="D59" t="n">
+        <v>714</v>
+      </c>
+      <c r="E59" t="n">
+        <v>4</v>
+      </c>
+      <c r="F59" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
A lot of stuff
</commit_message>
<xml_diff>
--- a/inputData/LTM_demand5min.xlsx
+++ b/inputData/LTM_demand5min.xlsx
@@ -465,19 +465,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -485,19 +485,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -505,19 +505,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -525,19 +525,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -545,19 +545,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -568,16 +568,16 @@
         <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D7" t="n">
-        <v>82</v>
+        <v>50</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -585,13 +585,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D8" t="n">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="E8" t="n">
         <v>2</v>
@@ -605,16 +605,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D9" t="n">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
@@ -625,13 +625,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D10" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E10" t="n">
         <v>4</v>
@@ -645,19 +645,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
         <v>9</v>
       </c>
-      <c r="C11" t="n">
-        <v>1</v>
-      </c>
       <c r="D11" t="n">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -665,16 +665,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C12" t="n">
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -685,13 +685,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D13" t="n">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="E13" t="n">
         <v>4</v>
@@ -705,19 +705,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -725,16 +725,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -745,16 +745,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C16" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>103</v>
+        <v>136</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
@@ -765,16 +765,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D17" t="n">
-        <v>108</v>
+        <v>140</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -785,19 +785,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>109</v>
+        <v>141</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -808,13 +808,13 @@
         <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D19" t="n">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -825,19 +825,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>111</v>
+        <v>152</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -845,16 +845,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>113</v>
+        <v>167</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
@@ -865,19 +865,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>116</v>
+        <v>170</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -885,19 +885,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>126</v>
+        <v>170</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -905,16 +905,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>141</v>
+        <v>173</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
@@ -928,16 +928,16 @@
         <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D25" t="n">
-        <v>147</v>
+        <v>180</v>
       </c>
       <c r="E25" t="n">
         <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -945,19 +945,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D26" t="n">
-        <v>148</v>
+        <v>188</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -971,13 +971,13 @@
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>150</v>
+        <v>188</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -985,16 +985,16 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
         <v>8</v>
       </c>
-      <c r="C28" t="n">
-        <v>7</v>
-      </c>
       <c r="D28" t="n">
-        <v>152</v>
+        <v>189</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1005,16 +1005,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>153</v>
+        <v>196</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1025,19 +1025,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>154</v>
+        <v>247</v>
       </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1045,16 +1045,16 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D31" t="n">
-        <v>156</v>
+        <v>253</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -1065,16 +1065,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
         <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>161</v>
+        <v>317</v>
       </c>
       <c r="E32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1085,16 +1085,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C33" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>172</v>
+        <v>369</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
@@ -1105,13 +1105,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D34" t="n">
-        <v>180</v>
+        <v>426</v>
       </c>
       <c r="E34" t="n">
         <v>4</v>
@@ -1125,19 +1125,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D35" t="n">
-        <v>186</v>
+        <v>436</v>
       </c>
       <c r="E35" t="n">
         <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1145,19 +1145,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>186</v>
+        <v>440</v>
       </c>
       <c r="E36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -1171,10 +1171,10 @@
         <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>189</v>
+        <v>469</v>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
@@ -1191,10 +1191,10 @@
         <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>204</v>
+        <v>473</v>
       </c>
       <c r="E38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -1211,7 +1211,7 @@
         <v>7</v>
       </c>
       <c r="D39" t="n">
-        <v>215</v>
+        <v>480</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -1228,16 +1228,16 @@
         <v>4</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D40" t="n">
-        <v>344</v>
+        <v>519</v>
       </c>
       <c r="E40" t="n">
         <v>4</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -1245,19 +1245,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>451</v>
+        <v>522</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -1265,19 +1265,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C42" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>480</v>
+        <v>526</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -1285,19 +1285,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>509</v>
+        <v>530</v>
       </c>
       <c r="E43" t="n">
         <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -1305,16 +1305,16 @@
         <v>43</v>
       </c>
       <c r="B44" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D44" t="n">
-        <v>510</v>
+        <v>548</v>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
@@ -1325,19 +1325,19 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D45" t="n">
-        <v>518</v>
+        <v>553</v>
       </c>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -1345,16 +1345,16 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C46" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>543</v>
+        <v>589</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -1371,13 +1371,13 @@
         <v>9</v>
       </c>
       <c r="D47" t="n">
-        <v>557</v>
+        <v>593</v>
       </c>
       <c r="E47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -1385,16 +1385,16 @@
         <v>47</v>
       </c>
       <c r="B48" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" t="n">
         <v>8</v>
       </c>
-      <c r="C48" t="n">
-        <v>7</v>
-      </c>
       <c r="D48" t="n">
-        <v>558</v>
+        <v>594</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
@@ -1405,13 +1405,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D49" t="n">
-        <v>561</v>
+        <v>596</v>
       </c>
       <c r="E49" t="n">
         <v>3</v>
@@ -1425,19 +1425,19 @@
         <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C50" t="n">
         <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>585</v>
+        <v>598</v>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -1448,13 +1448,13 @@
         <v>1</v>
       </c>
       <c r="C51" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D51" t="n">
-        <v>591</v>
+        <v>602</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F51" t="n">
         <v>1</v>
@@ -1465,16 +1465,16 @@
         <v>51</v>
       </c>
       <c r="B52" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>595</v>
+        <v>619</v>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
@@ -1491,13 +1491,13 @@
         <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>604</v>
+        <v>628</v>
       </c>
       <c r="E53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1505,16 +1505,16 @@
         <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C54" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>622</v>
+        <v>633</v>
       </c>
       <c r="E54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -1525,16 +1525,16 @@
         <v>54</v>
       </c>
       <c r="B55" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D55" t="n">
-        <v>625</v>
+        <v>662</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
@@ -1545,19 +1545,19 @@
         <v>55</v>
       </c>
       <c r="B56" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C56" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D56" t="n">
-        <v>627</v>
+        <v>673</v>
       </c>
       <c r="E56" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -1568,13 +1568,13 @@
         <v>1</v>
       </c>
       <c r="C57" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D57" t="n">
-        <v>642</v>
+        <v>678</v>
       </c>
       <c r="E57" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -1585,16 +1585,16 @@
         <v>57</v>
       </c>
       <c r="B58" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C58" t="n">
         <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>702</v>
+        <v>697</v>
       </c>
       <c r="E58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
@@ -1611,7 +1611,7 @@
         <v>7</v>
       </c>
       <c r="D59" t="n">
-        <v>714</v>
+        <v>752</v>
       </c>
       <c r="E59" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
Fix and improve heurtistc
</commit_message>
<xml_diff>
--- a/inputData/LTM_demand5min.xlsx
+++ b/inputData/LTM_demand5min.xlsx
@@ -471,10 +471,10 @@
         <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -485,13 +485,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -505,13 +505,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>45</v>
+        <v>101</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -525,19 +525,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
         <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -551,7 +551,7 @@
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>50</v>
+        <v>122</v>
       </c>
       <c r="E6" t="n">
         <v>3</v>
@@ -565,16 +565,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>133</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -585,16 +585,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>145</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
@@ -605,16 +605,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>84</v>
+        <v>150</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
@@ -625,13 +625,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10" t="n">
-        <v>85</v>
+        <v>154</v>
       </c>
       <c r="E10" t="n">
         <v>4</v>
@@ -645,16 +645,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>87</v>
+        <v>159</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -665,19 +665,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>92</v>
+        <v>168</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -685,19 +685,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D13" t="n">
-        <v>115</v>
+        <v>171</v>
       </c>
       <c r="E13" t="n">
         <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -705,16 +705,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>118</v>
+        <v>172</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
@@ -725,13 +725,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>120</v>
+        <v>178</v>
       </c>
       <c r="E15" t="n">
         <v>4</v>
@@ -745,13 +745,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>136</v>
+        <v>192</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
@@ -765,19 +765,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C17" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>140</v>
+        <v>195</v>
       </c>
       <c r="E17" t="n">
         <v>4</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -785,16 +785,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D18" t="n">
-        <v>141</v>
+        <v>263</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
@@ -808,16 +808,16 @@
         <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>143</v>
+        <v>303</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -825,19 +825,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>152</v>
+        <v>344</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -845,16 +845,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>167</v>
+        <v>390</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
@@ -865,19 +865,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D22" t="n">
-        <v>170</v>
+        <v>418</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -885,19 +885,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>170</v>
+        <v>430</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -905,19 +905,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D24" t="n">
-        <v>173</v>
+        <v>484</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -925,19 +925,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>180</v>
+        <v>497</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -945,19 +945,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D26" t="n">
-        <v>188</v>
+        <v>497</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -968,13 +968,13 @@
         <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>188</v>
+        <v>501</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -985,13 +985,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C28" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D28" t="n">
-        <v>189</v>
+        <v>504</v>
       </c>
       <c r="E28" t="n">
         <v>2</v>
@@ -1005,16 +1005,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C29" t="n">
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>196</v>
+        <v>509</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1025,16 +1025,16 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D30" t="n">
-        <v>247</v>
+        <v>510</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
@@ -1048,16 +1048,16 @@
         <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D31" t="n">
-        <v>253</v>
+        <v>516</v>
       </c>
       <c r="E31" t="n">
         <v>4</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1065,19 +1065,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D32" t="n">
-        <v>317</v>
+        <v>523</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -1085,16 +1085,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>369</v>
+        <v>535</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
@@ -1108,16 +1108,16 @@
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D34" t="n">
-        <v>426</v>
+        <v>542</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -1125,19 +1125,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>436</v>
+        <v>549</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1148,16 +1148,16 @@
         <v>7</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D36" t="n">
-        <v>440</v>
+        <v>552</v>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1165,19 +1165,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C37" t="n">
         <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>469</v>
+        <v>563</v>
       </c>
       <c r="E37" t="n">
         <v>4</v>
       </c>
       <c r="F37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1185,19 +1185,19 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C38" t="n">
         <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>473</v>
+        <v>567</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -1208,10 +1208,10 @@
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D39" t="n">
-        <v>480</v>
+        <v>570</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -1225,16 +1225,16 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C40" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>519</v>
+        <v>578</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
         <v>1</v>
@@ -1245,19 +1245,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>522</v>
+        <v>579</v>
       </c>
       <c r="E41" t="n">
         <v>3</v>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -1265,16 +1265,16 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D42" t="n">
-        <v>526</v>
+        <v>583</v>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -1285,19 +1285,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>530</v>
+        <v>594</v>
       </c>
       <c r="E43" t="n">
         <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -1308,10 +1308,10 @@
         <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D44" t="n">
-        <v>548</v>
+        <v>612</v>
       </c>
       <c r="E44" t="n">
         <v>1</v>
@@ -1325,16 +1325,16 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C45" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>553</v>
+        <v>617</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
@@ -1345,19 +1345,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C46" t="n">
         <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>589</v>
+        <v>629</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1368,16 +1368,16 @@
         <v>1</v>
       </c>
       <c r="C47" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
-        <v>593</v>
+        <v>629</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -1385,19 +1385,19 @@
         <v>47</v>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>594</v>
+        <v>646</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -1405,13 +1405,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C49" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D49" t="n">
-        <v>596</v>
+        <v>647</v>
       </c>
       <c r="E49" t="n">
         <v>3</v>
@@ -1425,16 +1425,16 @@
         <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C50" t="n">
         <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>598</v>
+        <v>649</v>
       </c>
       <c r="E50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F50" t="n">
         <v>1</v>
@@ -1445,16 +1445,16 @@
         <v>50</v>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C51" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D51" t="n">
-        <v>602</v>
+        <v>653</v>
       </c>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F51" t="n">
         <v>1</v>
@@ -1465,13 +1465,13 @@
         <v>51</v>
       </c>
       <c r="B52" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C52" t="n">
         <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>619</v>
+        <v>661</v>
       </c>
       <c r="E52" t="n">
         <v>2</v>
@@ -1485,19 +1485,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" t="n">
-        <v>628</v>
+        <v>662</v>
       </c>
       <c r="E53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -1505,13 +1505,13 @@
         <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C54" t="n">
         <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>633</v>
+        <v>712</v>
       </c>
       <c r="E54" t="n">
         <v>4</v>
@@ -1525,19 +1525,19 @@
         <v>54</v>
       </c>
       <c r="B55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C55" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>662</v>
+        <v>713</v>
       </c>
       <c r="E55" t="n">
         <v>4</v>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -1545,19 +1545,19 @@
         <v>55</v>
       </c>
       <c r="B56" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C56" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>673</v>
+        <v>716</v>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -1568,16 +1568,16 @@
         <v>1</v>
       </c>
       <c r="C57" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D57" t="n">
-        <v>678</v>
+        <v>733</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -1585,16 +1585,16 @@
         <v>57</v>
       </c>
       <c r="B58" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D58" t="n">
-        <v>697</v>
+        <v>740</v>
       </c>
       <c r="E58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
@@ -1605,19 +1605,19 @@
         <v>58</v>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C59" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>752</v>
+        <v>745</v>
       </c>
       <c r="E59" t="n">
         <v>4</v>
       </c>
       <c r="F59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>